<commit_message>
Complete revised portfolio construction and fix chart normalization
- Fill Candidates sheet: 15 stocks screened across 5 sectors, 5 selected
- Fill InheritedFund sheet: keep/drop decisions and target weights for all 10 legacy stocks
- Set active rule to optimizer/max_sharpe in Constraints sheet
- Fix legacy fund growth-of-$1 normalization in backtest charts (portfolio_utils.py, dashboard_app.py)
- Add capstone_requirements.txt for local venv setup outside iCloud
- Exclude data/raw/ from git (large ephemeral downloads)
- Update cached clean price panel with all 25 tickers

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fund_manager_control.xlsx
+++ b/fund_manager_control.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InheritedFund" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidates" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Constraints" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outputs" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes_Manifest" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="InheritedFund" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Candidates" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Constraints" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Outputs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Notes_Manifest" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -150,7 +150,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -234,6 +234,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -643,8 +644,8 @@
     <col width="58.33203125" customWidth="1" style="2" min="1" max="1"/>
     <col width="35.83203125" customWidth="1" style="2" min="2" max="2"/>
     <col width="26.6640625" customWidth="1" style="2" min="3" max="3"/>
-    <col width="10.83203125" customWidth="1" style="2" min="4" max="5"/>
-    <col width="10.83203125" customWidth="1" style="2" min="6" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="2" min="4" max="9"/>
+    <col width="10.83203125" customWidth="1" style="2" min="10" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -886,8 +887,8 @@
     <col width="20" customWidth="1" style="2" min="4" max="4"/>
     <col width="21.1640625" bestFit="1" customWidth="1" style="2" min="5" max="5"/>
     <col width="20" customWidth="1" style="2" min="6" max="9"/>
-    <col width="10.83203125" customWidth="1" style="2" min="10" max="11"/>
-    <col width="10.83203125" customWidth="1" style="2" min="12" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="2" min="10" max="15"/>
+    <col width="10.83203125" customWidth="1" style="2" min="16" max="16384"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -961,6 +962,19 @@
           <t>Technology</t>
         </is>
       </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" s="31" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -986,6 +1000,19 @@
           <t>Consumer Discretionary</t>
         </is>
       </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" s="31" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1011,6 +1038,19 @@
           <t>Financials</t>
         </is>
       </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Drop</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" s="31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1036,6 +1076,19 @@
           <t>Communication Services</t>
         </is>
       </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" s="31" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1061,6 +1114,19 @@
           <t>Communication Services</t>
         </is>
       </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H8" s="31" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1086,6 +1152,19 @@
           <t>Consumer Staples</t>
         </is>
       </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Drop</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1111,6 +1190,19 @@
           <t>Technology</t>
         </is>
       </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H10" s="31" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1136,6 +1228,19 @@
           <t>Technology</t>
         </is>
       </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Drop</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1161,6 +1266,19 @@
           <t>Financials</t>
         </is>
       </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Drop</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1185,6 +1303,19 @@
         <is>
           <t>Energy</t>
         </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Drop</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" s="31" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1206,12 +1337,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J28"/>
+  <dimension ref="A3:J18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="20" customWidth="1" style="2" min="1" max="10"/>
-    <col width="10.83203125" customWidth="1" style="2" min="11" max="12"/>
-    <col width="10.83203125" customWidth="1" style="2" min="13" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="2" min="11" max="16"/>
+    <col width="10.83203125" customWidth="1" style="2" min="17" max="16384"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -1269,175 +1400,750 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>AAA</t>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Financials / Payments</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Global cashless payment network with near-monopoly economics; secular shift from cash to digital payments</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Passes all 4 screens; network effect moat; best-in-class by 5yr EPS growth and network volume ($8.8T processed in 2019)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Selected: largest global payment network, highest EPS growth in sector</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BBB</t>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Financials / Payments</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Second-largest global payment network with economics nearly identical to Visa</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Passes all 4 screens; network effect moat; rejected by best-in-class sub-rule — V processed $8.8T vs MA $6.5T in 2019; larger network wins</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Rejected: passes all rules but loses best-in-class to V on network volume and EPS growth</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Financials / Payments</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Largest U.S. bank by assets with diversified financial services across retail, investment banking, and asset management</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Passes size and profitability screens; strong moat; rejected — traditional banking adds credit-cycle and regulatory risk; prefer pure-play payment network for 30-40yr horizon</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Rejected: moat present but banking model adds macro sensitivity inconsistent with fund mandate</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>DDD</t>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Recession-proof retailer with cost-advantage moat and active e-commerce pivot underway as of Jan 2020</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Passes all 4 screens; cost advantage + brand moat; best-in-class by global scale, revenue size, and 40+ yr dividend growth track record</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Selected: largest global retailer, superior scale moat, longest dividend growth streak in sector</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>EEE</t>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Membership-model warehouse retailer with exceptional customer loyalty and high annual renewal rates (~90%)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Passes all 4 screens; membership moat is strong; rejected by best-in-class sub-rule — WMT has larger global footprint and longer dividend growth history</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Rejected: strong candidate but loses best-in-class to WMT on scale and dividend track record</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>FFF</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Target Corporation</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Mid-size U.S. retailer with strong private-label brands and improving same-store sales momentum entering 2020</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Fails size screen — market cap ~$44B in Jan 2020, below $50B threshold; eliminated at first filter before reaching moat or growth analysis</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Rejected: fails Rule 1 (size) — market cap below $50B minimum as of Jan 2020</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>GGG</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CVX</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CVX</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Chevron Corporation</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Best-balance-sheet integrated oil major; oil demand on 2020 consensus was decades from structural peak</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Passes all 4 screens; regulatory license + scale moat; best-in-class vs. XOM on D/E ratio and credit strength; lower financial risk</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Selected: integrated major with superior balance sheet; best-in-class by debt-to-equity vs. XOM</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>HHH</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Largest U.S. integrated oil major; held in legacy inherited fund before manager takeover</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Passes size and profitability screens; regulatory license moat; rejected by best-in-class sub-rule — higher D/E ratio and weaker balance sheet than CVX as of Jan 2020</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Rejected: passes all rules but loses best-in-class to CVX on balance sheet strength</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>III</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ConocoPhillips</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Large U.S. exploration and production company focused solely on upstream oil and gas</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Passes size screen; fails moat screen — E&amp;P-only model has no downstream diversification, making returns more directly tied to spot commodity prices with no margin buffer</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Rejected: fails Rule 3 (moat) — no integrated buffer; commodity price exposure too high for retirement mandate</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>KKK</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NEE</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NEE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>NextEra Energy Inc.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Regulated Florida utility monopoly and worlds largest wind/solar operator; rare utility with 8-10% 5yr EPS CAGR as of 2020</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Passes all 4 screens; regulatory license moat; best-in-class by 5yr EPS CAGR (8-10% vs. 2-3% for DUK/SO/AEP); lowest coal exposure</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Selected: only utility combining regulated monopoly moat with meaningful EPS growth; renewable secular tailwind</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>LLL</t>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DUK</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DUK</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Duke Energy Corporation</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Large regulated utility serving 7.7M customers across the Southeast and Midwest U.S.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Passes size and profitability screens; regulatory license moat; rejected by best-in-class sub-rule — 5yr EPS CAGR ~2-3% vs NEE 8-10%; heavy coal generation fleet limits long-horizon growth</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Rejected: passes all rules but loses best-in-class to NEE on EPS growth and renewable positioning</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>MMM</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Southern Company</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Regulated utility serving the Southeast with a long dividend history and stable regulated earnings</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Passes size and profitability screens; regulatory license moat; rejected by best-in-class sub-rule — similar low EPS growth to DUK; slow renewable transition relative to NEE</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Rejected: passes all rules but loses best-in-class to NEE on EPS growth rate and forward-looking energy mix</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>NNN</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Inc.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Largest U.S. health insurer plus Optum data and pharmacy arm; aging demographics provide 30-40yr secular tailwind</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Passes all 4 screens; switching cost + network moat; best-in-class by 5yr EPS CAGR (~15%+ vs. peers at 6-8%); investment-grade balance sheet</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Selected: highest EPS growth in healthcare; switching cost moat from employer contracts; Optum diversification</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>OOO</t>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Diversified healthcare conglomerate spanning pharmaceuticals, medical devices, and consumer products</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Passes all 4 screens; brand + IP moat is strong; rejected by best-in-class sub-rule — 5yr EPS CAGR ~6-8% vs UNH 15%+; also facing active talc litigation headwinds as of Jan 2020</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Rejected: strong moat but lower EPS growth; litigation risk adds uncertainty inconsistent with retirement mandate</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>PPP</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>RRR</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>SSS</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>TTT</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>UUU</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>VVV</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>WWW</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>YYY</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>ZZZ</t>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CVS</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CVS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CVS Health Corporation</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Integrated pharmacy and insurance company following the 2018 Aetna acquisition</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Passes size and profitability screens; moderate switching cost moat; rejected — elevated D/E ratio from Aetna acquisition (2018) disqualifies under investment-grade requirement of best-in-class sub-rule</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Rejected: fails best-in-class sub-rule on balance sheet — Aetna debt load elevated D/E above acceptable threshold</t>
         </is>
       </c>
     </row>
@@ -1466,8 +2172,8 @@
     <col width="26.6640625" customWidth="1" style="2" min="1" max="1"/>
     <col width="15" customWidth="1" style="7" min="2" max="2"/>
     <col width="19.1640625" customWidth="1" style="2" min="3" max="3"/>
-    <col width="10.83203125" customWidth="1" style="2" min="4" max="5"/>
-    <col width="10.83203125" customWidth="1" style="2" min="6" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="2" min="4" max="9"/>
+    <col width="10.83203125" customWidth="1" style="2" min="10" max="16384"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -1617,7 +2323,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>equal_weight</t>
+          <t>optimizer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1678,18 +2384,18 @@
     <col width="18" customWidth="1" min="4" max="6"/>
     <col width="28" customWidth="1" style="2" min="7" max="7"/>
     <col width="24" customWidth="1" style="2" min="8" max="8"/>
-    <col width="14" customWidth="1" style="2" min="9" max="10"/>
-    <col width="14" customWidth="1" style="2" min="11" max="16384"/>
+    <col width="14" customWidth="1" style="2" min="9" max="14"/>
+    <col width="14" customWidth="1" style="2" min="15" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="31" t="inlineStr">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>Run Status</t>
         </is>
       </c>
-      <c r="B1" s="32" t="n"/>
-      <c r="C1" s="32" t="n"/>
+      <c r="B1" s="33" t="n"/>
+      <c r="C1" s="33" t="n"/>
       <c r="D1" s="8" t="n"/>
       <c r="E1" s="8" t="n"/>
       <c r="F1" s="8" t="n"/>
@@ -1728,7 +2434,7 @@
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
@@ -1774,7 +2480,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>OK: required sheets, parameters, columns, and price-panel quality checks were validated. Warnings: 1</t>
+          <t>OK: required sheets, parameters, columns, and price-panel quality checks were validated.</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
@@ -1797,7 +2503,7 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>PARTIAL: inherited-fund and candidate-screen outputs are ready; revised-static and revised-active are still pending.</t>
+          <t>YES: inherited-fund, candidate-screen, revised-static, revised-active, factor/regression, and scenario/stress CSVs/figures were exported successfully.</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
@@ -1836,17 +2542,17 @@
       <c r="I7" s="14" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="31" t="inlineStr">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>Final Portfolio Snapshot</t>
         </is>
       </c>
-      <c r="B8" s="32" t="n"/>
-      <c r="C8" s="32" t="n"/>
-      <c r="D8" s="32" t="n"/>
-      <c r="E8" s="32" t="n"/>
-      <c r="F8" s="32" t="n"/>
-      <c r="G8" s="32" t="n"/>
+      <c r="B8" s="33" t="n"/>
+      <c r="C8" s="33" t="n"/>
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="33" t="n"/>
+      <c r="F8" s="33" t="n"/>
+      <c r="G8" s="33" t="n"/>
       <c r="H8" s="8" t="n"/>
       <c r="I8" s="8" t="n"/>
     </row>
@@ -1902,7 +2608,7 @@
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>Legacy hold</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
@@ -1911,16 +2617,12 @@
         </is>
       </c>
       <c r="E10" s="17" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G10" s="18" t="inlineStr">
-        <is>
-          <t>Starter default: legacy equal-weight fund.</t>
-        </is>
-      </c>
+        <v>0.1471274389793825</v>
+      </c>
+      <c r="G10" s="18" t="inlineStr"/>
       <c r="H10" s="14" t="n"/>
       <c r="I10" s="14" t="n"/>
     </row>
@@ -1937,7 +2639,7 @@
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>Legacy hold</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
@@ -1946,23 +2648,19 @@
         </is>
       </c>
       <c r="E11" s="17" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G11" s="18" t="inlineStr">
-        <is>
-          <t>Starter default: legacy equal-weight fund.</t>
-        </is>
-      </c>
+        <v>0.1508812989850544</v>
+      </c>
+      <c r="G11" s="18" t="inlineStr"/>
       <c r="H11" s="14" t="n"/>
       <c r="I11" s="14" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>BRK-B</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
@@ -1972,7 +2670,7 @@
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>Legacy hold</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
@@ -1984,20 +2682,16 @@
         <v>0.1</v>
       </c>
       <c r="F12" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G12" s="18" t="inlineStr">
-        <is>
-          <t>Starter default: legacy equal-weight fund.</t>
-        </is>
-      </c>
+        <v>0.106404989268606</v>
+      </c>
+      <c r="G12" s="18" t="inlineStr"/>
       <c r="H12" s="14" t="n"/>
       <c r="I12" s="14" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
@@ -2007,7 +2701,7 @@
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>Legacy hold</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
@@ -2019,20 +2713,16 @@
         <v>0.1</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G13" s="18" t="inlineStr">
-        <is>
-          <t>Starter default: legacy equal-weight fund.</t>
-        </is>
-      </c>
+        <v>0.1017972584376416</v>
+      </c>
+      <c r="G13" s="18" t="inlineStr"/>
       <c r="H13" s="14" t="n"/>
       <c r="I13" s="14" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
@@ -2042,7 +2732,7 @@
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>Legacy hold</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
@@ -2054,30 +2744,26 @@
         <v>0.1</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G14" s="18" t="inlineStr">
-        <is>
-          <t>Starter default: legacy equal-weight fund.</t>
-        </is>
-      </c>
+        <v>0.1000609001022294</v>
+      </c>
+      <c r="G14" s="18" t="inlineStr"/>
       <c r="H14" s="14" t="n"/>
       <c r="I14" s="14" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>Inherited</t>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>Legacy hold</t>
+          <t>Add</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
@@ -2086,14 +2772,14 @@
         </is>
       </c>
       <c r="E15" s="17" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>0.1</v>
+        <v>0.08457226388181856</v>
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>Starter default: legacy equal-weight fund.</t>
+          <t>Selected: largest global payment network, highest EPS growth in sector</t>
         </is>
       </c>
       <c r="H15" s="14" t="n"/>
@@ -2102,17 +2788,17 @@
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>Inherited</t>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>Legacy hold</t>
+          <t>Add</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
@@ -2121,14 +2807,14 @@
         </is>
       </c>
       <c r="E16" s="17" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="F16" s="17" t="n">
-        <v>0.1</v>
+        <v>0.08393035349059123</v>
       </c>
       <c r="G16" s="18" t="inlineStr">
         <is>
-          <t>Starter default: legacy equal-weight fund.</t>
+          <t>Selected: largest global retailer, superior scale moat, longest dividend growth streak in sector</t>
         </is>
       </c>
       <c r="H16" s="14" t="n"/>
@@ -2137,17 +2823,17 @@
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>Inherited</t>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>Legacy hold</t>
+          <t>Add</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
@@ -2156,14 +2842,14 @@
         </is>
       </c>
       <c r="E17" s="17" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="F17" s="17" t="n">
-        <v>0.1</v>
+        <v>0.07665445186007529</v>
       </c>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>Starter default: legacy equal-weight fund.</t>
+          <t>Selected: integrated major with superior balance sheet; best-in-class by debt-to-equity vs. XOM</t>
         </is>
       </c>
       <c r="H17" s="14" t="n"/>
@@ -2172,17 +2858,17 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>WFC</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>Inherited</t>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>Legacy hold</t>
+          <t>Add</t>
         </is>
       </c>
       <c r="D18" s="16" t="inlineStr">
@@ -2191,14 +2877,14 @@
         </is>
       </c>
       <c r="E18" s="17" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="F18" s="17" t="n">
-        <v>0.1</v>
+        <v>0.07197041622530083</v>
       </c>
       <c r="G18" s="18" t="inlineStr">
         <is>
-          <t>Starter default: legacy equal-weight fund.</t>
+          <t>Selected: only utility combining regulated monopoly moat with meaningful EPS growth; renewable secular tailwind</t>
         </is>
       </c>
       <c r="H18" s="14" t="n"/>
@@ -2207,17 +2893,17 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>Inherited</t>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>Legacy hold</t>
+          <t>Add</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr">
@@ -2226,14 +2912,14 @@
         </is>
       </c>
       <c r="E19" s="17" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="F19" s="17" t="n">
-        <v>0.1</v>
+        <v>0.07660062876930029</v>
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>Starter default: legacy equal-weight fund.</t>
+          <t>Selected: highest EPS growth in healthcare; switching cost moat from employer contracts; Optum diversification</t>
         </is>
       </c>
       <c r="H19" s="14" t="n"/>
@@ -2251,19 +2937,19 @@
       <c r="I20" s="14" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="A21" s="32" t="inlineStr">
         <is>
           <t>Top-Level Performance Summary</t>
         </is>
       </c>
-      <c r="B21" s="32" t="n"/>
-      <c r="C21" s="32" t="n"/>
-      <c r="D21" s="32" t="n"/>
-      <c r="E21" s="32" t="n"/>
-      <c r="F21" s="32" t="n"/>
-      <c r="G21" s="32" t="n"/>
-      <c r="H21" s="32" t="n"/>
-      <c r="I21" s="32" t="n"/>
+      <c r="B21" s="33" t="n"/>
+      <c r="C21" s="33" t="n"/>
+      <c r="D21" s="33" t="n"/>
+      <c r="E21" s="33" t="n"/>
+      <c r="F21" s="33" t="n"/>
+      <c r="G21" s="33" t="n"/>
+      <c r="H21" s="33" t="n"/>
+      <c r="I21" s="33" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
@@ -2319,25 +3005,25 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>15261597.03215112</v>
+        <v>15261596.96739008</v>
       </c>
       <c r="C23" s="17" t="n">
-        <v>1.75709488454291</v>
+        <v>1.757094603014801</v>
       </c>
       <c r="D23" s="17" t="n">
-        <v>0.1846862191688263</v>
+        <v>0.1846861989538795</v>
       </c>
       <c r="E23" s="17" t="n">
-        <v>0.2432814255138178</v>
+        <v>0.2432813945947335</v>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.7591464033012936</v>
+        <v>0.75914641668976</v>
       </c>
       <c r="G23" s="21" t="n">
-        <v>1.002197819259307</v>
+        <v>1.002197876885282</v>
       </c>
       <c r="H23" s="17" t="n">
-        <v>-0.3137782372352629</v>
+        <v>-0.3137782669699901</v>
       </c>
       <c r="I23" s="17" t="n">
         <v>0</v>
@@ -2349,14 +3035,30 @@
           <t>Revised Static Fund</t>
         </is>
       </c>
-      <c r="B24" s="20" t="n"/>
-      <c r="C24" s="17" t="n"/>
-      <c r="D24" s="17" t="n"/>
-      <c r="E24" s="17" t="n"/>
-      <c r="F24" s="21" t="n"/>
-      <c r="G24" s="21" t="n"/>
-      <c r="H24" s="17" t="n"/>
-      <c r="I24" s="17" t="n"/>
+      <c r="B24" s="20" t="n">
+        <v>14048737.59742697</v>
+      </c>
+      <c r="C24" s="17" t="n">
+        <v>1.537984635015615</v>
+      </c>
+      <c r="D24" s="17" t="n">
+        <v>0.168405655926855</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>0.2190818660371811</v>
+      </c>
+      <c r="F24" s="21" t="n">
+        <v>0.76868824870368</v>
+      </c>
+      <c r="G24" s="21" t="n">
+        <v>0.9819216569586509</v>
+      </c>
+      <c r="H24" s="17" t="n">
+        <v>-0.273907482893831</v>
+      </c>
+      <c r="I24" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
@@ -2364,14 +3066,30 @@
           <t>Revised Active Fund</t>
         </is>
       </c>
-      <c r="B25" s="20" t="n"/>
-      <c r="C25" s="17" t="n"/>
-      <c r="D25" s="17" t="n"/>
-      <c r="E25" s="17" t="n"/>
-      <c r="F25" s="21" t="n"/>
-      <c r="G25" s="21" t="n"/>
-      <c r="H25" s="17" t="n"/>
-      <c r="I25" s="17" t="n"/>
+      <c r="B25" s="20" t="n">
+        <v>14100074.20713302</v>
+      </c>
+      <c r="C25" s="17" t="n">
+        <v>1.547258886580511</v>
+      </c>
+      <c r="D25" s="17" t="n">
+        <v>0.1691180541192125</v>
+      </c>
+      <c r="E25" s="17" t="n">
+        <v>0.2133341758305466</v>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>0.7927377479993858</v>
+      </c>
+      <c r="G25" s="21" t="n">
+        <v>1.004152961658763</v>
+      </c>
+      <c r="H25" s="17" t="n">
+        <v>-0.27829229113173</v>
+      </c>
+      <c r="I25" s="17" t="n">
+        <v>0.02146566493433784</v>
+      </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
@@ -2380,25 +3098,25 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>12679565.90321468</v>
+        <v>12679565.84077461</v>
       </c>
       <c r="C26" s="17" t="n">
-        <v>1.290636177611785</v>
+        <v>1.290635942153882</v>
       </c>
       <c r="D26" s="17" t="n">
-        <v>0.1485550554107495</v>
+        <v>0.1485550356816079</v>
       </c>
       <c r="E26" s="17" t="n">
-        <v>0.207413144776657</v>
+        <v>0.2074130727806035</v>
       </c>
       <c r="F26" s="21" t="n">
-        <v>0.7162277760684552</v>
+        <v>0.7162279295613433</v>
       </c>
       <c r="G26" s="21" t="n">
-        <v>0.8802486710270973</v>
+        <v>0.8802491213900754</v>
       </c>
       <c r="H26" s="17" t="n">
-        <v>-0.3371725334437184</v>
+        <v>-0.3371726482138072</v>
       </c>
       <c r="I26" s="17" t="n">
         <v>0</v>
@@ -2427,13 +3145,13 @@
       <c r="I28" s="14" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="31" t="inlineStr">
+      <c r="A29" s="32" t="inlineStr">
         <is>
           <t>Active Rule / Implementation Summary</t>
         </is>
       </c>
-      <c r="B29" s="32" t="n"/>
-      <c r="C29" s="32" t="n"/>
+      <c r="B29" s="33" t="n"/>
+      <c r="C29" s="33" t="n"/>
       <c r="D29" s="8" t="n"/>
       <c r="E29" s="8" t="n"/>
       <c r="F29" s="8" t="n"/>
@@ -2472,7 +3190,7 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>equal_weight</t>
+          <t>sharpe_tilt</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
@@ -2581,12 +3299,12 @@
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>No active rebalances have been executed yet.</t>
+          <t>Latest effective rebalance date. Average monthly turnover=2.1%.</t>
         </is>
       </c>
       <c r="D36" s="14" t="n"/>
@@ -2603,7 +3321,7 @@
         </is>
       </c>
       <c r="B37" s="24" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
@@ -2618,17 +3336,17 @@
       <c r="I37" s="14" t="n"/>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="31" t="inlineStr">
+      <c r="A38" s="32" t="inlineStr">
         <is>
           <t>Factor / Regression Snapshot</t>
         </is>
       </c>
-      <c r="B38" s="32" t="n"/>
-      <c r="C38" s="32" t="n"/>
-      <c r="D38" s="32" t="n"/>
-      <c r="E38" s="32" t="n"/>
-      <c r="F38" s="32" t="n"/>
-      <c r="G38" s="32" t="n"/>
+      <c r="B38" s="33" t="n"/>
+      <c r="C38" s="33" t="n"/>
+      <c r="D38" s="33" t="n"/>
+      <c r="E38" s="33" t="n"/>
+      <c r="F38" s="33" t="n"/>
+      <c r="G38" s="33" t="n"/>
       <c r="H38" s="8" t="n"/>
       <c r="I38" s="8" t="n"/>
     </row>
@@ -2678,16 +3396,16 @@
         </is>
       </c>
       <c r="B40" s="17" t="n">
-        <v>0.0316350346175087</v>
+        <v>0.03163500163955029</v>
       </c>
       <c r="C40" s="21" t="n">
-        <v>1.064890557876907</v>
+        <v>1.064890883453683</v>
       </c>
       <c r="D40" s="17" t="n">
-        <v>0.8235779435905095</v>
+        <v>0.8235780804314634</v>
       </c>
       <c r="E40" s="21" t="n">
-        <v>83.84716818334908</v>
+        <v>83.84720766698554</v>
       </c>
       <c r="F40" s="26" t="n">
         <v>0</v>
@@ -2701,24 +3419,60 @@
       <c r="I40" s="14" t="n"/>
     </row>
     <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="16" t="n"/>
-      <c r="B41" s="17" t="n"/>
-      <c r="C41" s="21" t="n"/>
-      <c r="D41" s="17" t="n"/>
-      <c r="E41" s="21" t="n"/>
-      <c r="F41" s="26" t="n"/>
-      <c r="G41" s="18" t="n"/>
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>Revised Static Fund</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="n">
+        <v>0.02164288998715659</v>
+      </c>
+      <c r="C41" s="21" t="n">
+        <v>0.9872216861302682</v>
+      </c>
+      <c r="D41" s="17" t="n">
+        <v>0.8735519992489141</v>
+      </c>
+      <c r="E41" s="21" t="n">
+        <v>102.0001671248496</v>
+      </c>
+      <c r="F41" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="18" t="inlineStr">
+        <is>
+          <t>latest rolling beta=0.85; proxy=benchmark_return; n=1508</t>
+        </is>
+      </c>
       <c r="H41" s="14" t="n"/>
       <c r="I41" s="14" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="16" t="n"/>
-      <c r="B42" s="17" t="n"/>
-      <c r="C42" s="21" t="n"/>
-      <c r="D42" s="17" t="n"/>
-      <c r="E42" s="21" t="n"/>
-      <c r="F42" s="26" t="n"/>
-      <c r="G42" s="18" t="n"/>
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>Revised Active Fund</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="n">
+        <v>0.02438337956065459</v>
+      </c>
+      <c r="C42" s="21" t="n">
+        <v>0.9661947118137731</v>
+      </c>
+      <c r="D42" s="17" t="n">
+        <v>0.8824308741621525</v>
+      </c>
+      <c r="E42" s="21" t="n">
+        <v>106.3178507695399</v>
+      </c>
+      <c r="F42" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="18" t="inlineStr">
+        <is>
+          <t>latest rolling beta=0.76; proxy=benchmark_return; n=1508</t>
+        </is>
+      </c>
       <c r="H42" s="14" t="n"/>
       <c r="I42" s="14" t="n"/>
     </row>
@@ -2745,18 +3499,18 @@
       <c r="I44" s="14" t="n"/>
     </row>
     <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="31" t="inlineStr">
+      <c r="A45" s="32" t="inlineStr">
         <is>
           <t>Scenario / Stress Snapshot</t>
         </is>
       </c>
-      <c r="B45" s="32" t="n"/>
-      <c r="C45" s="32" t="n"/>
-      <c r="D45" s="32" t="n"/>
-      <c r="E45" s="32" t="n"/>
-      <c r="F45" s="32" t="n"/>
-      <c r="G45" s="32" t="n"/>
-      <c r="H45" s="32" t="n"/>
+      <c r="B45" s="33" t="n"/>
+      <c r="C45" s="33" t="n"/>
+      <c r="D45" s="33" t="n"/>
+      <c r="E45" s="33" t="n"/>
+      <c r="F45" s="33" t="n"/>
+      <c r="G45" s="33" t="n"/>
+      <c r="H45" s="33" t="n"/>
       <c r="I45" s="8" t="n"/>
     </row>
     <row r="46" ht="24" customHeight="1">
@@ -2808,15 +3562,29 @@
           <t>Revised Static Fund</t>
         </is>
       </c>
-      <c r="B47" s="17" t="n"/>
-      <c r="C47" s="17" t="n"/>
-      <c r="D47" s="17" t="n"/>
-      <c r="E47" s="17" t="n"/>
-      <c r="F47" s="16" t="inlineStr"/>
-      <c r="G47" s="17" t="n"/>
+      <c r="B47" s="17" t="n">
+        <v>0.1920325280450351</v>
+      </c>
+      <c r="C47" s="17" t="n">
+        <v>-0.1789012724756603</v>
+      </c>
+      <c r="D47" s="17" t="n">
+        <v>0.1651544991206367</v>
+      </c>
+      <c r="E47" s="17" t="n">
+        <v>0.6470241075079166</v>
+      </c>
+      <c r="F47" s="16" t="inlineStr">
+        <is>
+          <t>Worst 21-Day Window</t>
+        </is>
+      </c>
+      <c r="G47" s="17" t="n">
+        <v>-0.2606477903046253</v>
+      </c>
       <c r="H47" s="18" t="inlineStr">
         <is>
-          <t>Scenario/stress outputs are not ready yet.</t>
+          <t>Uses compounded selected-universe returns over the worst 21-day benchmark-proxy window.</t>
         </is>
       </c>
       <c r="I47" s="14" t="n"/>
@@ -2827,15 +3595,29 @@
           <t>Revised Active Fund</t>
         </is>
       </c>
-      <c r="B48" s="17" t="n"/>
-      <c r="C48" s="17" t="n"/>
-      <c r="D48" s="17" t="n"/>
-      <c r="E48" s="17" t="n"/>
-      <c r="F48" s="16" t="inlineStr"/>
-      <c r="G48" s="17" t="n"/>
+      <c r="B48" s="17" t="n">
+        <v>0.1995608752366695</v>
+      </c>
+      <c r="C48" s="17" t="n">
+        <v>-0.1650178054773065</v>
+      </c>
+      <c r="D48" s="17" t="n">
+        <v>0.167962322171559</v>
+      </c>
+      <c r="E48" s="17" t="n">
+        <v>0.6680095974678362</v>
+      </c>
+      <c r="F48" s="16" t="inlineStr">
+        <is>
+          <t>Worst 21-Day Window</t>
+        </is>
+      </c>
+      <c r="G48" s="17" t="n">
+        <v>-0.2581813390473018</v>
+      </c>
       <c r="H48" s="18" t="inlineStr">
         <is>
-          <t>Scenario/stress outputs are not ready yet.</t>
+          <t>Uses compounded selected-universe returns over the worst 21-day benchmark-proxy window.</t>
         </is>
       </c>
       <c r="I48" s="14" t="n"/>
@@ -2896,13 +3678,13 @@
       <c r="I53" s="14" t="n"/>
     </row>
     <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="31" t="inlineStr">
+      <c r="A54" s="32" t="inlineStr">
         <is>
           <t>Major Artifacts</t>
         </is>
       </c>
-      <c r="B54" s="32" t="n"/>
-      <c r="C54" s="32" t="n"/>
+      <c r="B54" s="33" t="n"/>
+      <c r="C54" s="33" t="n"/>
       <c r="D54" s="8" t="n"/>
       <c r="E54" s="8" t="n"/>
       <c r="F54" s="8" t="n"/>
@@ -2964,12 +3746,12 @@
       </c>
       <c r="B57" s="16" t="inlineStr">
         <is>
-          <t>fig_backtest_legacy_vs_benchmark.png</t>
+          <t>fig_legacy_static_active_benchmark.png</t>
         </is>
       </c>
       <c r="C57" s="16" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_backtest_legacy_vs_benchmark.png</t>
+          <t>outputs/figures/fig_legacy_static_active_benchmark.png</t>
         </is>
       </c>
       <c r="D57" s="14" t="n"/>
@@ -2987,12 +3769,12 @@
       </c>
       <c r="B58" s="16" t="inlineStr">
         <is>
-          <t>fig_candidate_risk_return.png</t>
+          <t>fig_legacy_static_benchmark.png</t>
         </is>
       </c>
       <c r="C58" s="16" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_candidate_risk_return.png</t>
+          <t>outputs/figures/fig_legacy_static_benchmark.png</t>
         </is>
       </c>
       <c r="D58" s="14" t="n"/>
@@ -3010,12 +3792,12 @@
       </c>
       <c r="B59" s="16" t="inlineStr">
         <is>
-          <t>fig_revised_static_weights.png</t>
+          <t>fig_backtest_legacy_vs_benchmark.png</t>
         </is>
       </c>
       <c r="C59" s="16" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_revised_static_weights.png</t>
+          <t>outputs/figures/fig_backtest_legacy_vs_benchmark.png</t>
         </is>
       </c>
       <c r="D59" s="14" t="n"/>
@@ -3033,12 +3815,12 @@
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>fig_factor_alpha_beta.png</t>
+          <t>fig_candidate_risk_return.png</t>
         </is>
       </c>
       <c r="C60" s="16" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_factor_alpha_beta.png</t>
+          <t>outputs/figures/fig_candidate_risk_return.png</t>
         </is>
       </c>
       <c r="D60" s="14" t="n"/>
@@ -3056,12 +3838,12 @@
       </c>
       <c r="B61" s="16" t="inlineStr">
         <is>
-          <t>fig_factor_rolling_beta.png</t>
+          <t>fig_revised_static_weights.png</t>
         </is>
       </c>
       <c r="C61" s="16" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_factor_rolling_beta.png</t>
+          <t>outputs/figures/fig_revised_static_weights.png</t>
         </is>
       </c>
       <c r="D61" s="14" t="n"/>
@@ -3079,12 +3861,12 @@
       </c>
       <c r="B62" s="16" t="inlineStr">
         <is>
-          <t>fig_scenario_monte_carlo_distribution.png</t>
+          <t>fig_revised_active_weights.png</t>
         </is>
       </c>
       <c r="C62" s="16" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_scenario_monte_carlo_distribution.png</t>
+          <t>outputs/figures/fig_revised_active_weights.png</t>
         </is>
       </c>
       <c r="D62" s="14" t="n"/>
@@ -3102,12 +3884,12 @@
       </c>
       <c r="B63" s="16" t="inlineStr">
         <is>
-          <t>fig_scenario_stress_impacts.png</t>
+          <t>fig_factor_alpha_beta.png</t>
         </is>
       </c>
       <c r="C63" s="16" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_scenario_stress_impacts.png</t>
+          <t>outputs/figures/fig_factor_alpha_beta.png</t>
         </is>
       </c>
       <c r="D63" s="14" t="n"/>
@@ -3120,17 +3902,17 @@
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="16" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>figure</t>
         </is>
       </c>
       <c r="B64" s="16" t="inlineStr">
         <is>
-          <t>tbl_backtest_legacy_static_active_benchmark.csv</t>
+          <t>fig_factor_rolling_beta.png</t>
         </is>
       </c>
       <c r="C64" s="16" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_backtest_legacy_static_active_benchmark.csv</t>
+          <t>outputs/figures/fig_factor_rolling_beta.png</t>
         </is>
       </c>
       <c r="D64" s="14" t="n"/>
@@ -3143,17 +3925,17 @@
     <row r="65" ht="20" customHeight="1">
       <c r="A65" s="16" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>figure</t>
         </is>
       </c>
       <c r="B65" s="16" t="inlineStr">
         <is>
-          <t>tbl_backtest_legacy_static_benchmark.csv</t>
+          <t>fig_scenario_monte_carlo_distribution.png</t>
         </is>
       </c>
       <c r="C65" s="16" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_backtest_legacy_static_benchmark.csv</t>
+          <t>outputs/figures/fig_scenario_monte_carlo_distribution.png</t>
         </is>
       </c>
       <c r="D65" s="14" t="n"/>
@@ -3166,17 +3948,17 @@
     <row r="66" ht="20" customHeight="1">
       <c r="A66" s="16" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>figure</t>
         </is>
       </c>
       <c r="B66" s="16" t="inlineStr">
         <is>
-          <t>tbl_backtest_legacy_vs_benchmark.csv</t>
+          <t>fig_scenario_stress_impacts.png</t>
         </is>
       </c>
       <c r="C66" s="16" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_backtest_legacy_vs_benchmark.csv</t>
+          <t>outputs/figures/fig_scenario_stress_impacts.png</t>
         </is>
       </c>
       <c r="D66" s="14" t="n"/>
@@ -3194,12 +3976,12 @@
       </c>
       <c r="B67" s="16" t="inlineStr">
         <is>
-          <t>tbl_factor_capm_summary.csv</t>
+          <t>tbl_backtest_legacy_static_active_benchmark.csv</t>
         </is>
       </c>
       <c r="C67" s="16" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_factor_capm_summary.csv</t>
+          <t>outputs/tables/tbl_backtest_legacy_static_active_benchmark.csv</t>
         </is>
       </c>
       <c r="D67" s="14" t="n"/>
@@ -3217,12 +3999,12 @@
       </c>
       <c r="B68" s="16" t="inlineStr">
         <is>
-          <t>tbl_scenario_stress_summary.csv</t>
+          <t>tbl_backtest_legacy_static_benchmark.csv</t>
         </is>
       </c>
       <c r="C68" s="16" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_scenario_stress_summary.csv</t>
+          <t>outputs/tables/tbl_backtest_legacy_static_benchmark.csv</t>
         </is>
       </c>
       <c r="D68" s="14" t="n"/>
@@ -3240,12 +4022,12 @@
       </c>
       <c r="B69" s="16" t="inlineStr">
         <is>
-          <t>tbl_project_manifest.csv</t>
+          <t>tbl_backtest_legacy_vs_benchmark.csv</t>
         </is>
       </c>
       <c r="C69" s="16" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_project_manifest.csv</t>
+          <t>outputs/tables/tbl_backtest_legacy_vs_benchmark.csv</t>
         </is>
       </c>
       <c r="D69" s="14" t="n"/>
@@ -3256,9 +4038,21 @@
       <c r="I69" s="14" t="n"/>
     </row>
     <row r="70" ht="20" customHeight="1">
-      <c r="A70" s="16" t="n"/>
-      <c r="B70" s="16" t="n"/>
-      <c r="C70" s="16" t="n"/>
+      <c r="A70" s="16" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="B70" s="16" t="inlineStr">
+        <is>
+          <t>tbl_factor_capm_summary.csv</t>
+        </is>
+      </c>
+      <c r="C70" s="16" t="inlineStr">
+        <is>
+          <t>outputs/tables/tbl_factor_capm_summary.csv</t>
+        </is>
+      </c>
       <c r="D70" s="14" t="n"/>
       <c r="E70" s="14" t="n"/>
       <c r="F70" s="14" t="n"/>
@@ -3267,9 +4061,21 @@
       <c r="I70" s="14" t="n"/>
     </row>
     <row r="71" ht="20" customHeight="1">
-      <c r="A71" s="16" t="n"/>
-      <c r="B71" s="16" t="n"/>
-      <c r="C71" s="16" t="n"/>
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="B71" s="16" t="inlineStr">
+        <is>
+          <t>tbl_scenario_stress_summary.csv</t>
+        </is>
+      </c>
+      <c r="C71" s="16" t="inlineStr">
+        <is>
+          <t>outputs/tables/tbl_scenario_stress_summary.csv</t>
+        </is>
+      </c>
       <c r="D71" s="14" t="n"/>
       <c r="E71" s="14" t="n"/>
       <c r="F71" s="14" t="n"/>
@@ -3278,9 +4084,21 @@
       <c r="I71" s="14" t="n"/>
     </row>
     <row r="72" ht="20" customHeight="1">
-      <c r="A72" s="16" t="n"/>
-      <c r="B72" s="16" t="n"/>
-      <c r="C72" s="16" t="n"/>
+      <c r="A72" s="16" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="B72" s="16" t="inlineStr">
+        <is>
+          <t>tbl_project_manifest.csv</t>
+        </is>
+      </c>
+      <c r="C72" s="16" t="inlineStr">
+        <is>
+          <t>outputs/tables/tbl_project_manifest.csv</t>
+        </is>
+      </c>
       <c r="D72" s="14" t="n"/>
       <c r="E72" s="14" t="n"/>
       <c r="F72" s="14" t="n"/>
@@ -3625,21 +4443,21 @@
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="10.83203125" customWidth="1" style="2" min="7" max="8"/>
-    <col width="10.83203125" customWidth="1" style="2" min="9" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="2" min="7" max="12"/>
+    <col width="10.83203125" customWidth="1" style="2" min="13" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="33" t="inlineStr">
+      <c r="A1" s="34" t="inlineStr">
         <is>
           <t>Notes and Manifest</t>
         </is>
       </c>
-      <c r="B1" s="32" t="n"/>
-      <c r="C1" s="32" t="n"/>
-      <c r="D1" s="32" t="n"/>
-      <c r="E1" s="32" t="n"/>
-      <c r="F1" s="32" t="n"/>
+      <c r="B1" s="33" t="n"/>
+      <c r="C1" s="33" t="n"/>
+      <c r="D1" s="33" t="n"/>
+      <c r="E1" s="33" t="n"/>
+      <c r="F1" s="33" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
@@ -3663,11 +4481,7 @@
           <t>known_issue_1</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>No revised 2020 portfolio selections detected yet. Pipeline will default to the legacy fund summary.</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3720,7 +4534,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3730,12 +4544,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>pipeline_20260417_095136.log</t>
+          <t>pipeline_20260424_105713.log</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>outputs/logs/pipeline_20260417_095136.log</t>
+          <t>outputs/logs/pipeline_20260424_105713.log</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3748,7 +4562,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3776,7 +4590,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3804,7 +4618,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3832,7 +4646,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3860,7 +4674,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3888,7 +4702,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3916,7 +4730,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3944,7 +4758,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3972,7 +4786,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4000,7 +4814,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4028,7 +4842,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4056,7 +4870,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4084,7 +4898,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4112,7 +4926,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4140,7 +4954,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4168,7 +4982,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4178,12 +4992,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>tbl_backtest_legacy_static_benchmark.csv</t>
+          <t>tbl_revised_static_weights_daily.csv</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_backtest_legacy_static_benchmark.csv</t>
+          <t>outputs/tables/tbl_revised_static_weights_daily.csv</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -4196,7 +5010,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4206,12 +5020,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>tbl_revised_active_daily.csv</t>
+          <t>tbl_revised_static_weights_snapshot.csv</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_revised_active_daily.csv</t>
+          <t>outputs/tables/tbl_revised_static_weights_snapshot.csv</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4224,7 +5038,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4234,12 +5048,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>tbl_revised_active_weights_daily.csv</t>
+          <t>tbl_backtest_legacy_static_benchmark.csv</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_revised_active_weights_daily.csv</t>
+          <t>outputs/tables/tbl_backtest_legacy_static_benchmark.csv</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -4252,7 +5066,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4262,12 +5076,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>tbl_revised_active_rebalance_log.csv</t>
+          <t>tbl_revised_active_daily.csv</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_revised_active_rebalance_log.csv</t>
+          <t>outputs/tables/tbl_revised_active_daily.csv</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -4280,7 +5094,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4290,12 +5104,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>tbl_backtest_legacy_static_active_benchmark.csv</t>
+          <t>tbl_revised_active_weights_daily.csv</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_backtest_legacy_static_active_benchmark.csv</t>
+          <t>outputs/tables/tbl_revised_active_weights_daily.csv</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4308,7 +5122,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4318,12 +5132,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>tbl_factor_capm_summary.csv</t>
+          <t>tbl_revised_active_weights_snapshot.csv</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_factor_capm_summary.csv</t>
+          <t>outputs/tables/tbl_revised_active_weights_snapshot.csv</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -4336,7 +5150,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4346,12 +5160,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>tbl_factor_rolling_beta.csv</t>
+          <t>tbl_revised_active_rebalance_log.csv</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_factor_rolling_beta.csv</t>
+          <t>outputs/tables/tbl_revised_active_rebalance_log.csv</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4364,7 +5178,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4374,12 +5188,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>tbl_scenario_monte_carlo_summary.csv</t>
+          <t>tbl_backtest_legacy_static_active_benchmark.csv</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_scenario_monte_carlo_summary.csv</t>
+          <t>outputs/tables/tbl_backtest_legacy_static_active_benchmark.csv</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4392,7 +5206,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4402,12 +5216,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>tbl_scenario_monte_carlo_draws.csv</t>
+          <t>tbl_factor_capm_summary.csv</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_scenario_monte_carlo_draws.csv</t>
+          <t>outputs/tables/tbl_factor_capm_summary.csv</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4420,7 +5234,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -4430,12 +5244,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>tbl_scenario_stress_summary.csv</t>
+          <t>tbl_factor_rolling_beta.csv</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>outputs/tables/tbl_scenario_stress_summary.csv</t>
+          <t>outputs/tables/tbl_factor_rolling_beta.csv</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4448,22 +5262,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>figure</t>
+          <t>table</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>fig_inherited_fund_overview.png</t>
+          <t>tbl_scenario_monte_carlo_summary.csv</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_inherited_fund_overview.png</t>
+          <t>outputs/tables/tbl_scenario_monte_carlo_summary.csv</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -4476,22 +5290,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>figure</t>
+          <t>table</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>fig_inherited_drawdown.png</t>
+          <t>tbl_scenario_monte_carlo_draws.csv</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_inherited_drawdown.png</t>
+          <t>outputs/tables/tbl_scenario_monte_carlo_draws.csv</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4504,22 +5318,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>figure</t>
+          <t>table</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>fig_inherited_weights_snapshot.png</t>
+          <t>tbl_scenario_stress_summary.csv</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_inherited_weights_snapshot.png</t>
+          <t>outputs/tables/tbl_scenario_stress_summary.csv</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4532,7 +5346,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -4542,12 +5356,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>fig_backtest_legacy_vs_benchmark.png</t>
+          <t>fig_inherited_fund_overview.png</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_backtest_legacy_vs_benchmark.png</t>
+          <t>outputs/figures/fig_inherited_fund_overview.png</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4560,7 +5374,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -4570,12 +5384,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>fig_candidate_risk_return.png</t>
+          <t>fig_inherited_drawdown.png</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_candidate_risk_return.png</t>
+          <t>outputs/figures/fig_inherited_drawdown.png</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -4588,7 +5402,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4598,12 +5412,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>fig_candidate_recent_return.png</t>
+          <t>fig_inherited_weights_snapshot.png</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_candidate_recent_return.png</t>
+          <t>outputs/figures/fig_inherited_weights_snapshot.png</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4616,7 +5430,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4626,12 +5440,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>fig_revised_static_weights.png</t>
+          <t>fig_backtest_legacy_vs_benchmark.png</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_revised_static_weights.png</t>
+          <t>outputs/figures/fig_backtest_legacy_vs_benchmark.png</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -4644,7 +5458,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -4654,12 +5468,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>fig_factor_alpha_beta.png</t>
+          <t>fig_candidate_risk_return.png</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_factor_alpha_beta.png</t>
+          <t>outputs/figures/fig_candidate_risk_return.png</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -4672,7 +5486,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -4682,12 +5496,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>fig_factor_rolling_beta.png</t>
+          <t>fig_candidate_recent_return.png</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_factor_rolling_beta.png</t>
+          <t>outputs/figures/fig_candidate_recent_return.png</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -4700,7 +5514,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -4710,12 +5524,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>fig_scenario_monte_carlo_distribution.png</t>
+          <t>fig_revised_static_weights.png</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_scenario_monte_carlo_distribution.png</t>
+          <t>outputs/figures/fig_revised_static_weights.png</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -4728,7 +5542,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -4738,12 +5552,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>fig_scenario_stress_impacts.png</t>
+          <t>fig_legacy_static_benchmark.png</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>outputs/figures/fig_scenario_stress_impacts.png</t>
+          <t>outputs/figures/fig_legacy_static_benchmark.png</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -4756,22 +5570,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>figure</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>yf_prices_raw_20260417_095138.csv</t>
+          <t>fig_revised_active_weights.png</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>data/raw/yf_prices_raw_20260417_095138.csv</t>
+          <t>outputs/figures/fig_revised_active_weights.png</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -4784,22 +5598,22 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>figure</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>prices_adjclose_daily.csv</t>
+          <t>fig_legacy_static_active_benchmark.png</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>data/clean/prices_adjclose_daily.csv</t>
+          <t>outputs/figures/fig_legacy_static_active_benchmark.png</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -4812,22 +5626,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>figure</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>returns_daily.csv</t>
+          <t>fig_factor_alpha_beta.png</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>data/clean/returns_daily.csv</t>
+          <t>outputs/figures/fig_factor_alpha_beta.png</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -4840,36 +5654,171 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-04-17 09:51:39</t>
+          <t>2026-04-24 10:57:15</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
+          <t>figure</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>fig_factor_rolling_beta.png</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>outputs/figures/fig_factor_rolling_beta.png</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>created</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:57:15</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>figure</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>fig_scenario_monte_carlo_distribution.png</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>outputs/figures/fig_scenario_monte_carlo_distribution.png</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>created</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:57:15</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>figure</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>fig_scenario_stress_impacts.png</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>outputs/figures/fig_scenario_stress_impacts.png</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>created</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:57:15</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
           <t>table</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>prices_adjclose_daily.csv</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>data/clean/prices_adjclose_daily.csv</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>created</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:57:15</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>returns_daily.csv</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>data/clean/returns_daily.csv</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>created</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:57:15</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
         <is>
           <t>tbl_project_manifest.csv</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>outputs/tables/tbl_project_manifest.csv</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>created</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
-    </row>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
+      <c r="F66" t="inlineStr"/>
+    </row>
     <row r="67"/>
     <row r="68"/>
     <row r="69"/>

</xml_diff>